<commit_message>
feat(core-math): M1 engine — namespaced RNG, integer accounting, exact+MC, CLI
- rng.rs: counter-based namespaced ChaCha8 (subsystem,spin,draw) [ADR-003]
- accounting.rs/stats.rs: integer/u128 money + streaming stats [ADR-002, ADR-012]
- mechanics.rs: LTR+wild line eval & scatter counting (shared by exact & MC)
- enumerate.rs: exact line+scatter RTP, uncapped [ADR-001]
- simulate.rs: deterministic Rayon Monte Carlo (thread-independent)
- bin/cli.rs: numeric math sheet; examples/sample_5x3.json reference game
- tests: determinism, exact==MC within CI, hand-verifiable 72/27 (6 green)

Reference game: exact 95.30% == MC within CI, ~19M spins/s. Stable v0.2.0 pending
external certified-game parity, cap-inside-exact-math, and weight-reels.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SaS-Math-AI_Features_and_Metrics.xlsx
+++ b/SaS-Math-AI_Features_and_Metrics.xlsx
@@ -38,7 +38,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -52,12 +52,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
+        <fgColor rgb="00FEF9C3"/>
       </patternFill>
     </fill>
   </fills>
@@ -87,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -100,6 +105,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -541,7 +549,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -578,7 +586,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -615,7 +623,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -652,7 +660,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -689,7 +697,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -726,7 +734,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -763,7 +771,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -800,7 +808,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -833,7 +841,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -864,7 +872,7 @@
           <t>optimize against the exact engine</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -901,7 +909,7 @@
           <t>variance reduction for MC parts</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -938,7 +946,7 @@
           <t>preserve positional/adjacency constraints</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -975,7 +983,7 @@
           <t>gameplay-shape targets as hard constraints</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1012,7 +1020,7 @@
           <t>contributions reconcile to the unit</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1049,7 +1057,7 @@
           <t>Rust core in-process to Python</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1086,7 +1094,7 @@
           <t>constrained decoding from fixed Lego library</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1123,7 +1131,7 @@
           <t>models generated from schema</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1160,7 +1168,7 @@
           <t>translate / validate / simulate / tune</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1193,7 +1201,7 @@
           <t>generated from schema; locks hard bounds</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1230,7 +1238,7 @@
           <t>raw config view / tweak</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1263,7 +1271,7 @@
           <t>store configs + results</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1300,7 +1308,7 @@
           <t>end-to-end tests</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1337,7 +1345,7 @@
           <t>cascades / expanding wilds / multipliers</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1374,7 +1382,7 @@
           <t>PDF/Excel certification math sheet</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1407,7 +1415,7 @@
           <t>on every Monte Carlo metric</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1511,7 +1519,11 @@
           <t>per design (e.g. 96.00)</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>95.30</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
           <t>%</t>
@@ -1544,7 +1556,11 @@
           <t>CI contains exact value</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>95.34 +/- 0.11</t>
+        </is>
+      </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>%</t>
@@ -1577,7 +1593,11 @@
           <t>per design (e.g. med-high)</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>2.47</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>sigma</t>
@@ -1610,7 +1630,11 @@
           <t>per design</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>51.33</t>
+        </is>
+      </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
           <t>%</t>
@@ -1742,7 +1766,11 @@
           <t>10M &lt; 2s (&gt;=5M/s)</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>~19M/s (10M in 0.55s)</t>
+        </is>
+      </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
           <t>spins/s</t>
@@ -1775,7 +1803,11 @@
           <t>50/50 identical to the unit</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>PASS (thread-independent)</t>
+        </is>
+      </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
           <t>pass/fail</t>
@@ -1808,7 +1840,11 @@
           <t>within CI</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>within 95% CI</t>
+        </is>
+      </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
           <t>%</t>
@@ -1841,7 +1877,11 @@
           <t>&lt; 0.001</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>pending external game</t>
+        </is>
+      </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
           <t>%</t>
@@ -2000,7 +2040,7 @@
           <t>clean documented checkpoint</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -2027,9 +2067,9 @@
           <t>Parity Test passes; seed-replay identical; 10M &lt; 2s</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2094,7 @@
           <t>broken 140% RTP config -&gt; fixed playable 96%</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -2081,7 +2121,7 @@
           <t>prompt -&gt; JSON -&gt; simulate -&gt; tune in browser</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -2108,7 +2148,7 @@
           <t>exported sheet matches a certified live game</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -2125,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2196,6 +2236,33 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>v0.2.0-beta.1</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>M1 core-math engine: namespaced RNG, integer accounting, exact+MC, CLI; 6 tests green (~19M spins/s)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>last stable = v0.1.0; git checkout v0.1.0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(core-math): exact cap fold-in + weight-reels [M1]
- enumerate.rs: exact capped RTP via column-tuple enumeration (min(win,cap) per atom),
  feasibility-bounded (ENUM_LIMIT) with numeric-MC fallback labeled by provenance;
  built-in cross-check that enumeration-uncapped == closed-form [ADR-005]
- mechanics.rs: weight-reels realized to deterministic spread strips [ADR-006];
  precomputed per-reel columns for enumeration
- config.rs: reels accept strips OR weights
- cli.rs: capped RTP + cap-erosion + provenance label
- tests: cap_fold_in_is_exact (40/27), enumeration==closed-form, weights==strips (9 green)

Sample 50x cap -> 0.057% exact cap-erosion over 33.5M combos; MC within CI.
Stable v0.2.0 still pending external certified-game parity.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SaS-Math-AI_Features_and_Metrics.xlsx
+++ b/SaS-Math-AI_Features_and_Metrics.xlsx
@@ -2165,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2263,6 +2263,33 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>v0.2.0-beta.2</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>M1 cont.: exact capped enumeration (cap-erosion) + weight-reels; provenance-labeled; 9 tests green</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>last stable = v0.1.0; git checkout v0.1.0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(solver): M2 auto-tuner — weight-tuning to target RTP + re-verify
- solver.rs: closed-form RTP as a smooth function of per-reel weights (line marginals
  + binomial scatter); (mu/mu_w,lambda)-ES with CSA step control (deterministic);
  bounds + light regularizer for non-degeneracy; realize tuned weights -> integer
  strips for re-verification [ADR-006]
- bin/tune.rs: load config + target RTP -> tune -> re-verify (exact+MC) -> write tuned config
- config: derive Serialize (write tuned configs); reels accept strips OR weights
- tests: closed-form line == engine; gate 139%->96% + re-verify; non-degenerate;
  deterministic solve (13 tests green)

Gate PASS: broken_lineonly 139.2% -> 95.9% (within 0.09%), realize-delta 0.02%,
hit-freq 42%->45%. Known follow-up: align engine weighted-reel scatter to the
solver's binomial model (scatter-only re-verify delta).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SaS-Math-AI_Features_and_Metrics.xlsx
+++ b/SaS-Math-AI_Features_and_Metrics.xlsx
@@ -2094,9 +2094,9 @@
           <t>broken 140% RTP config -&gt; fixed playable 96%</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2290,6 +2290,33 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>v0.3.0-beta.1</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>M2 auto-tuner: ES weight-tuning to target RTP + realize/re-verify; gate PASS 139%-&gt;96% line game; 13 tests green</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>last stable = v0.1.0; git checkout v0.1.0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(M2): scatter-consistent engine + multi-objective solver
- mechanics: explicit ReelModel{Strips,Weights}. Weights now independent-cell
  (binomial scatter + independent-cell MC) instead of realized-to-strip, so the
  solver objective and re-verify use the SAME model. Scatter re-verify delta 5.8% -> 0.3%.
- enumerate: unified line marginal (sym_count/reel_size); scatter branched
  (Strips window / Weights binomial); cap enumeration Strips-only.
- simulate: MC branches on model (stops vs independent-cell draws).
- solver: shared run_es core; solve_multi + SolveTargets tune RTP + volatility +
  hit-frequency (RTP exact closed-form; vol/hit via CRN Monte Carlo). tune CLI
  takes [target_vol] [target_hit].
- tests: weighted exact scatter == MC; scatter game re-verifies; multi-objective
  hits RTP + volatility (16 green).

Demo: vol 4.0->4.029 (hit 29%) and 2.0->1.970 (36%) at ~96% RTP.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SaS-Math-AI_Features_and_Metrics.xlsx
+++ b/SaS-Math-AI_Features_and_Metrics.xlsx
@@ -2165,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2317,6 +2317,33 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>v0.3.0-beta.2</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>M2 finished: scatter-consistent (independent-cell) + multi-objective (RTP+vol+hit); scatter re-verify delta 5.8%-&gt;0.3%; 16 tests green</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>last stable = v0.1.0; git checkout v0.1.0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(M3): AI layer — FastAPI translator + Rust JSON engine bridge
- core-math/src/bin/engine.rs: JSON stdin/stdout bridge (simulate|tune) so Python
  drives the engine/solver without PyO3. Also changed pays/weights map keys to
  String (internally-tagged serde enums buffer content and break integer map keys).
- ai-layer (FastAPI + Pydantic 2): models.py (schema mirror), mechanics.py (fixed
  library + base-config builder), translator.py (rule-based provider-agnostic
  translator + provider stub, ADR-008), engine.py (subprocess bridge), main.py
  (/translate /validate /simulate /tune /design /health).
- 6 pytest green. Gate: POST /design runs prompt->JSON->simulate->tune;
  '5x3, 20 lines, 96% RTP, medium vol, wild+scatter' -> 1.49 -> 0.9600 RTP, delta 0.0001.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SaS-Math-AI_Features_and_Metrics.xlsx
+++ b/SaS-Math-AI_Features_and_Metrics.xlsx
@@ -2121,9 +2121,9 @@
           <t>prompt -&gt; JSON -&gt; simulate -&gt; tune in browser</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2344,6 +2344,33 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>v0.4.0-beta.1</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>M3 ai-layer: FastAPI + provider-agnostic translator + Rust JSON engine bridge; prompt-&gt;JSON-&gt;simulate-&gt;tune pipeline; 6 Python tests</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>last stable = v0.1.0; git checkout v0.1.0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(M3): Next.js Slot Studio frontend (browser-verified)
- frontend/: Next.js 16 + React 19 + Tailwind v4 + Zustand + Monaco
  - app/page.tsx: prompt -> Monaco config -> Simulate/Tune (RTP/vol/hit cards)
  - lib/api.ts: typed ai-layer client; store/useStore.ts: Zustand state
- ai-layer: CORS for the browser origin
- Browser-verified (preview tools): Translate 200 -> Simulate 149.19% -> Auto-tune 96.00%
  (realize-delta 0.01%); next build type-checks clean.

M3 'in browser' gate met: prompt -> JSON -> simulate -> tune.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SaS-Math-AI_Features_and_Metrics.xlsx
+++ b/SaS-Math-AI_Features_and_Metrics.xlsx
@@ -2165,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2371,6 +2371,33 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>v0.4.0-beta.2</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>M3 frontend: Next.js Slot Studio (Tailwind/Zustand/Monaco); browser-verified prompt-&gt;translate-&gt;simulate-&gt;tune 149%-&gt;96%</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>last stable = v0.1.0; git checkout v0.1.0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>